<commit_message>
Basic implementation of an InProcessQueue and passing TransactionItem into Process
</commit_message>
<xml_diff>
--- a/Data/Config_Dev.xlsx
+++ b/Data/Config_Dev.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{549F1927-F52B-437D-AE6E-A1BD6463E64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5079B62-6B5A-4B36-A79F-CF51191C7408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1230" yWindow="3720" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1575" yWindow="4065" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="63">
   <si>
     <t>Name</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>.\Data\Temp\ACME</t>
+  </si>
+  <si>
+    <t>Target_Batchsize</t>
   </si>
 </sst>
 </file>
@@ -589,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1003"/>
+  <dimension ref="A1:Z1005"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -704,99 +707,106 @@
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" t="s">
-        <v>39</v>
+        <v>62</v>
+      </c>
+      <c r="B13" s="5">
+        <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="5">
-        <v>10</v>
-      </c>
-    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>44</v>
+        <v>34</v>
+      </c>
+      <c r="B16" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A22" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="5">
-        <v>21</v>
-      </c>
-    </row>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="B24" s="5">
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A27" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B27" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
@@ -1773,6 +1783,8 @@
     <row r="1001" ht="14.25" customHeight="1"/>
     <row r="1002" ht="14.25" customHeight="1"/>
     <row r="1003" ht="14.25" customHeight="1"/>
+    <row r="1004" ht="14.25" customHeight="1"/>
+    <row r="1005" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactored code was split into workflows, needs argument cleansing. Added parsing of rpachallenge success message.
</commit_message>
<xml_diff>
--- a/Data/Config_Dev.xlsx
+++ b/Data/Config_Dev.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D0E388-36FA-4D6D-8677-6F2499CF8405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF43B446-B6DA-42C9-8955-810F2269CA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
   <si>
     <t>Name</t>
   </si>
@@ -223,6 +223,15 @@
   </si>
   <si>
     <t>False</t>
+  </si>
+  <si>
+    <t>Mailbox_FolderSuccessfulFormatA</t>
+  </si>
+  <si>
+    <t>Mailbox_FolderSuccessfulFormatB</t>
+  </si>
+  <si>
+    <t>RPA/PurposefulPromethium/successful/oldWay</t>
   </si>
 </sst>
 </file>
@@ -601,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1005"/>
+  <dimension ref="A1:Z1007"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -744,97 +753,111 @@
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>40</v>
+        <v>63</v>
+      </c>
+      <c r="B17" s="5">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A20" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A23" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>49</v>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A22" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
+    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="5">
-        <v>21</v>
+        <v>60</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A25" t="s">
-        <v>47</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
+    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>52</v>
+        <v>45</v>
+      </c>
+      <c r="B27" s="5">
+        <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="5">
-        <v>0</v>
+        <v>51</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -1808,6 +1831,8 @@
     <row r="1003" ht="14.25" customHeight="1"/>
     <row r="1004" ht="14.25" customHeight="1"/>
     <row r="1005" ht="14.25" customHeight="1"/>
+    <row r="1006" ht="14.25" customHeight="1"/>
+    <row r="1007" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Implemented EndToEnd test case.
</commit_message>
<xml_diff>
--- a/Data/Config_Dev.xlsx
+++ b/Data/Config_Dev.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF43B446-B6DA-42C9-8955-810F2269CA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0381C18F-6290-4A1C-86E5-8AFBE7AEE78C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1095" yWindow="3540" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="71">
   <si>
     <t>Name</t>
   </si>
@@ -232,6 +232,12 @@
   </si>
   <si>
     <t>RPA/PurposefulPromethium/successful/oldWay</t>
+  </si>
+  <si>
+    <t>The current count when populating the batch</t>
+  </si>
+  <si>
+    <t>The count desired for rpachallenge.com</t>
   </si>
 </sst>
 </file>
@@ -283,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -294,6 +300,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -730,6 +740,9 @@
       <c r="B13" s="5">
         <v>10</v>
       </c>
+      <c r="C13" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -751,15 +764,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A17" t="s">
+    <row r="17" spans="1:3" s="6" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A17" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="7">
         <v>0</v>
       </c>
+      <c r="C17" s="6" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+    <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -767,7 +783,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="14.25" customHeight="1">
+    <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -775,7 +791,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="14.25" customHeight="1">
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -783,7 +799,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="14.25" customHeight="1">
+    <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -791,7 +807,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="14.25" customHeight="1">
+    <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -799,8 +815,8 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:2" ht="14.25" customHeight="1">
+    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
         <v>60</v>
       </c>
@@ -808,8 +824,8 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:2" ht="14.25" customHeight="1">
+    <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
         <v>46</v>
       </c>
@@ -817,7 +833,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1">
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
         <v>45</v>
       </c>
@@ -825,7 +841,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="14.25" customHeight="1">
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
         <v>47</v>
       </c>
@@ -833,7 +849,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="14.25" customHeight="1">
+    <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -841,7 +857,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="14.25" customHeight="1">
+    <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
         <v>51</v>
       </c>
@@ -849,8 +865,8 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1">
+    <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
         <v>64</v>
       </c>

</xml_diff>

<commit_message>
Implemented InProcessQueue retry mechanism
</commit_message>
<xml_diff>
--- a/Data/Config_Dev.xlsx
+++ b/Data/Config_Dev.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0381C18F-6290-4A1C-86E5-8AFBE7AEE78C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070FF6CA-1ECB-440F-8C2E-A284C6974F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1095" yWindow="3540" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1095" yWindow="3540" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -1907,7 +1907,7 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Migrated to targetFramework Windows
- Test cases updated and pass without issue
- Automation executes end-to-end in Studio 2025.0.x Community Edition targeting Windows
- Project.json updated with "targetFramework": "Windows"
</commit_message>
<xml_diff>
--- a/Data/Config_Dev.xlsx
+++ b/Data/Config_Dev.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070FF6CA-1ECB-440F-8C2E-A284C6974F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576850CA-B7CF-4022-B037-F5AF0CADB1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1095" yWindow="3540" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9900" yWindow="2715" windowWidth="18270" windowHeight="11670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -117,9 +117,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>wildduck.email</t>
-  </si>
-  <si>
     <t>Imap_Server</t>
   </si>
   <si>
@@ -238,6 +235,9 @@
   </si>
   <si>
     <t>The count desired for rpachallenge.com</t>
+  </si>
+  <si>
+    <t>mail.wildduck.email</t>
   </si>
 </sst>
 </file>
@@ -308,7 +308,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -324,7 +324,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -621,7 +621,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z1007"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
     <col min="2" max="2" width="43" style="5" customWidth="1"/>
@@ -676,10 +676,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -689,7 +689,7 @@
         <v>26</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>29</v>
@@ -698,27 +698,27 @@
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" t="s">
         <v>56</v>
-      </c>
-      <c r="C7" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="5" t="s">
         <v>30</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="5">
         <v>993</v>
@@ -726,39 +726,39 @@
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13" s="5">
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B16" s="5">
         <v>2</v>
@@ -766,76 +766,76 @@
     </row>
     <row r="17" spans="1:3" s="6" customFormat="1" ht="14.25" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B17" s="7">
         <v>0</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B27" s="5">
         <v>21</v>
@@ -843,35 +843,35 @@
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>47</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1"/>
@@ -1859,7 +1859,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
@@ -2967,7 +2967,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
     <col min="2" max="2" width="30.140625" customWidth="1"/>

</xml_diff>

<commit_message>
breaking: finalized migration to targetFramework Windows
</commit_message>
<xml_diff>
--- a/Data/Config_Dev.xlsx
+++ b/Data/Config_Dev.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070FF6CA-1ECB-440F-8C2E-A284C6974F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7F4DF36-F049-4846-9287-4761362F3DB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1095" yWindow="3540" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="13500" windowHeight="21285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -117,9 +117,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>wildduck.email</t>
-  </si>
-  <si>
     <t>Imap_Server</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>OrchestratorFolderPath</t>
   </si>
   <si>
-    <t>ChapterEvents</t>
-  </si>
-  <si>
     <t>File_BasePathTemp</t>
   </si>
   <si>
@@ -238,6 +232,12 @@
   </si>
   <si>
     <t>The count desired for rpachallenge.com</t>
+  </si>
+  <si>
+    <t>rpapub</t>
+  </si>
+  <si>
+    <t>mail.wildduck.email</t>
   </si>
 </sst>
 </file>
@@ -676,10 +676,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -689,7 +689,7 @@
         <v>26</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>29</v>
@@ -698,27 +698,27 @@
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" t="s">
         <v>56</v>
-      </c>
-      <c r="C7" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="5">
         <v>993</v>
@@ -726,39 +726,39 @@
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B13" s="5">
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B16" s="5">
         <v>2</v>
@@ -766,76 +766,76 @@
     </row>
     <row r="17" spans="1:3" s="6" customFormat="1" ht="14.25" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B17" s="7">
         <v>0</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B27" s="5">
         <v>21</v>
@@ -843,35 +843,35 @@
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>47</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1"/>

</xml_diff>